<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.002-06 Les bateaux de la cour
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.002-06.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.002-06.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aniss veut faire courir ses bateaux de papier dans la flaque de la cour. Chouchou regarde, puis dit plus tard. Aniss accepte, dégage le bateau d'une feuille, et les deux sèchent sur le rebord.</t>
+          <t>L'air froid glisse le long du zinc. Sur une dalle, un éclat de dalle brille. Aniss veut faire courir les bateaux jusqu'à l'éclat, maintenant. Il propose. Chouchou regarde, puis dit plus tard. Le bateau s'arrête sur une feuille. Sourire parti. Aniss refuse de foncer, accepte, dégage le bateau. Merci vécu. Deux bateaux trop vite : ils se cognent. L'éclat de dalle tient au bout de la flaque.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le zinc de la gouttière sent le métal froid. Une goutte tombe encore. Elle fait un rond dans la flaque. Les dalles de la cour sont sombres. Un escargot avance sur une fissure. Ça sent la pierre mouillée. Maman pose un torchon sur le rebord. Tu as vu l'escargot, Aniss ? Oui, maman. Il a une petite maison. Oui. On le laisse tout doux. Deux bateaux de papier attendent. Ils sont un peu froissés. Papa les a pliés ce matin. Ils peuvent flotter dans la flaque. Je veux les faire courir. Le long des dalles ? Oui. En ce moment, Aniss pose un bateau. Le papier devient sombre. Il boit un peu d'eau. Il part ! Tout doux. Chouchou est sur la marche sèche. Ses chaussettes restent au sec. Aniss le voit. Tu viens ? On fait courir les bateaux. Je regarde. Aniss écoute. D'accord. On peut proposer. Tu as proposé, Aniss. Aniss pousse le bateau du doigt. Le bateau glisse entre deux dalles. L'escargot s'écarte, tout lent. Il laisse passer ! Oui. Une feuille collée barre le chemin. Le bateau s'arrête. Il est coincé. Tu peux le dégager. Aniss cherche autour de la flaque. Il regarde Chouchou. Tu m'aides ? Plus tard. D'accord. La feuille est juste devant. Le zinc goutte encore une fois. Le rond tremble, puis s'arrête.</t>
+          <t>L'air froid glisse le long du zinc. Aniss connaît cette cour, ses dalles, le bruit de la gouttière. Un détail paraît nouveau, sur une dalle sombre. Au bout de la flaque, un éclat de dalle brille. Il brille, papa. Tu le vois, sur la dalle ? Oui, tout au bout. Ça sent la pierre mouillée. Maman pose un torchon sur le rebord. Tu as vu l'éclat, Aniss ? Oui, maman. Deux bateaux de papier attendent. Ils sont un peu froissés. Papa les a pliés, ce matin. Ils peuvent flotter dans la flaque. Je veux les faire courir, maintenant ! Jusqu'à l'éclat, le long des dalles. Le long des dalles ? Oui, maman. Un escargot avance sur une fissure. Il a une petite maison. On le laisse sur sa fissure ? Oui, papa. Chouchou est sur la marche sèche. Ses chaussettes restent au sec. Elle tient le torchon, près du rebord. Tu as le torchon, Chouchou ? Oui, maman. Aniss le voit, sur la marche. Tu viens ? On fait courir les bateaux. Chouchou penche la tête. Elle ne descend pas. Je regarde. Aniss écoute. D'accord. En ce moment, Aniss pose un bateau. Le papier devient sombre. Il boit un peu d'eau. Il part ! Aniss pousse trop vite, du doigt. Le bateau glisse entre deux dalles. L'escargot s'écarte, très lent. Il laisse passer ! Une feuille collée barre le chemin. Le bateau s'arrête, loin de l'éclat. Il est coincé ! Il n'arrive pas au bout. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. L'éclat de dalle tremble, puis tient. Les épaules d'Aniss tombent un peu. Papa se baisse à sa hauteur. Tu vois la feuille ? Oui, papa. Aniss cherche autour de la flaque. Il regarde Chouchou. Tu m'aides ? Chouchou serre le torchon. Elle reste sur la marche. Plus tard. Aniss ouvre la bouche. Puis il la referme. Ça serre, dans son ventre.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le zinc de la gouttière sent le métal froid. Une goutte tombe encore. Elle fait un rond dans la flaque. Les dalles de la cour sont sombres. Un escargot avance sur une fissure. Ça sent la pierre mouillée. Maman pose un torchon sur le rebord. Tu as vu l'escargot, Aniss ? Oui, maman. Il a une petite maison. Oui. On le laisse tout doux. Deux bateaux de papier attendent. Ils sont un peu froissés. Papa les a pliés ce matin. Ils peuvent flotter dans la flaque. Je veux les faire courir. Le long des dalles ? Oui. En ce moment, Aniss pose un bateau. Le papier devient sombre. Il boit un peu d'eau. Il part ! Tout doux. Chouchou est sur la marche sèche. Ses chaussettes restent au sec. Aniss le voit. Tu viens ? On fait courir les bateaux. Je regarde. Aniss écoute. D'accord. On peut proposer. Tu as proposé, Aniss. Aniss pousse le bateau du doigt. Le bateau glisse entre deux dalles. L'escargot s'écarte, tout lent. Il laisse passer ! Oui. Une feuille collée barre le chemin. Le bateau s'arrête. Il est coincé. Tu peux le dégager. Aniss cherche autour de la flaque. Il regarde Chouchou. Tu m'aides ? Plus tard. D'accord. La feuille est juste devant. Le zinc goutte encore une fois. Le rond tremble, puis s'arrête.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'air froid glisse le long du zinc. Aniss connaît cette cour, ses dalles, le bruit de la gouttière. Un détail paraît nouveau, sur une dalle sombre. Au bout de la flaque, un &lt;emphasis level="moderate"&gt;éclat de dalle&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur la dalle ? Oui, tout au bout. Ça sent la pierre mouillée. Maman pose un torchon sur le rebord. Tu as vu l'éclat, Aniss ? Oui, maman. Deux bateaux de papier attendent. Ils sont un peu froissés. Papa les a pliés, ce matin. Ils peuvent flotter dans la flaque. Je veux les faire courir, maintenant ! Jusqu'à l'éclat, le long des dalles. Le long des dalles ? Oui, maman. Un escargot avance sur une fissure. Il a une petite maison. On le laisse sur sa fissure ? Oui, papa. Chouchou est sur la marche sèche. Ses chaussettes restent au sec. Elle tient le torchon, près du rebord. Tu as le torchon, Chouchou ? Oui, maman. Aniss le voit, sur la marche. Tu viens ? On fait courir les bateaux. Chouchou penche la tête. Elle ne descend pas. Je regarde. Aniss écoute. D'accord. En ce moment, Aniss pose un bateau. Le papier devient sombre. Il boit un peu d'eau. Il part ! Aniss pousse trop vite, du doigt. Le bateau glisse entre deux dalles. L'escargot s'écarte, très lent. Il laisse passer ! Une feuille collée barre le chemin. Le bateau s'arrête, loin de l'éclat. Il est coincé ! Il n'arrive pas au bout. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. L'éclat de dalle tremble, puis tient. Les épaules d'Aniss tombent un peu. Papa se baisse à sa hauteur. Tu vois la feuille ? Oui, papa. Aniss cherche autour de la flaque. Il regarde Chouchou. Tu m'aides ? Chouchou serre le torchon. Elle reste sur la marche. Plus tard. Aniss ouvre la bouche. Puis il la referme. Ça serre, dans son ventre.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Solal est au parc avec maman. Maëlys est près du bac. Solal va &lt;emphasis&gt;proposer&lt;/emphasis&gt; le seau. Il dit : tu viens ? Maëlys dit : je regarde. Solal accepte. Maman dit : on peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. Solal creuse. Maëlys regarde. Solal propose encore, tout doux : plus tard ? Maëlys dit : plus tard. Solal dit : d'accord. [pause]</t>
+          <t>L'air froid glisse le long du zinc. Aniss connaît cette cour, ses dalles, le bruit de la gouttière. Un détail paraît nouveau, sur une dalle sombre. Au bout de la flaque, un &lt;emphasis&gt;éclat de dalle&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur la dalle ? Oui, tout au bout. Ça sent la pierre mouillée. Maman pose un torchon sur le rebord. Tu as vu l'éclat, Aniss ? Oui, maman. Deux bateaux de papier attendent. Ils sont un peu froissés. Papa les a pliés, ce matin. Ils peuvent flotter dans la flaque. Je veux les faire courir, maintenant ! Jusqu'à l'éclat, le long des dalles. Le long des dalles ? Oui, maman. Un escargot avance sur une fissure. Il a une petite maison. On le laisse sur sa fissure ? Oui, papa. Chouchou est sur la marche sèche. Ses chaussettes restent au sec. Elle tient le torchon, près du rebord. Tu as le torchon, Chouchou ? Oui, maman. Aniss le voit, sur la marche. Tu viens ? On fait courir les bateaux. Chouchou penche la tête. Elle ne descend pas. Je regarde. Aniss écoute. D'accord. En ce moment, Aniss pose un bateau. Le papier devient sombre. Il boit un peu d'eau. Il part ! Aniss pousse trop vite, du doigt. Le bateau glisse entre deux dalles. L'escargot s'écarte, très lent. Il laisse passer ! Une feuille collée barre le chemin. Le bateau s'arrête, loin de l'éclat. Il est coincé ! Il n'arrive pas au bout. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. L'éclat de dalle tremble, puis tient. Les épaules d'Aniss tombent un peu. Papa se baisse à sa hauteur. Tu vois la feuille ? Oui, papa. Aniss cherche autour de la flaque. Il regarde Chouchou. Tu m'aides ? Chouchou serre le torchon. Elle reste sur la marche. Plus tard. Aniss ouvre la bouche. Puis il la referme. Ça serre, dans son ventre. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>éclat de dalle</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,65 +1326,82 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_les_bateaux_jusqu_a_l_eclat_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le zinc de la gouttière sent le métal froid.
-narrateur|Une goutte tombe encore.
-narrateur|Elle fait un rond dans la flaque.
-narrateur|Les dalles de la cour sont sombres.
-narrateur|Un escargot avance sur une fissure.
+          <t>narrateur|L'air froid glisse le long du zinc.
+narrateur|Aniss connaît cette cour, ses dalles, le bruit de la gouttière.
+narrateur|Un détail paraît nouveau, sur une dalle sombre.
+narrateur|Au bout de la flaque, un éclat de dalle brille.
+enfant-m|Il brille, papa.
+papa|Tu le vois, sur la dalle ?
+enfant-m|Oui, tout au bout.
 narrateur|Ça sent la pierre mouillée.
 narrateur|Maman pose un torchon sur le rebord.
-maman|Tu as vu l'escargot, Aniss ?
+maman|Tu as vu l'éclat, Aniss ?
 enfant-m|Oui, maman.
-enfant-m|Il a une petite maison.
-maman|Oui.
-maman|On le laisse tout doux.
 narrateur|Deux bateaux de papier attendent.
 narrateur|Ils sont un peu froissés.
-narrateur|Papa les a pliés ce matin.
+narrateur|Papa les a pliés, ce matin.
 papa|Ils peuvent flotter dans la flaque.
-enfant-m|Je veux les faire courir.
+enfant-m|Je veux les faire courir, maintenant !
+enfant-m|Jusqu'à l'éclat, le long des dalles.
 maman|Le long des dalles ?
-enfant-m|Oui.
+enfant-m|Oui, maman.
+narrateur|Un escargot avance sur une fissure.
+enfant-m|Il a une petite maison.
+papa|On le laisse sur sa fissure ?
+enfant-m|Oui, papa.
+narrateur|Chouchou est sur la marche sèche.
+narrateur|Ses chaussettes restent au sec.
+narrateur|Elle tient le torchon, près du rebord.
+maman|Tu as le torchon, Chouchou ?
+enfant-f|Oui, maman.
+narrateur|Aniss le voit, sur la marche.
+enfant-m|Tu viens ?
+enfant-m|On fait courir les bateaux.
+narrateur|Chouchou penche la tête.
+narrateur|Elle ne descend pas.
+enfant-f|Je regarde.
+narrateur|Aniss écoute.
+enfant-m|D'accord.
 narrateur|En ce moment, Aniss pose un bateau.
 narrateur|Le papier devient sombre.
 narrateur|Il boit un peu d'eau.
 enfant-m|Il part !
-maman|Tout doux.
-narrateur|Chouchou est sur la marche sèche.
-narrateur|Ses chaussettes restent au sec.
-narrateur|Aniss le voit.
-enfant-m|Tu viens ?
-enfant-m|On fait courir les bateaux.
-copain|Je regarde.
-narrateur|Aniss écoute.
-enfant-m|D'accord.
-maman|On peut proposer.
-maman|Tu as proposé, Aniss.
-narrateur|Aniss pousse le bateau du doigt.
+narrateur|Aniss pousse trop vite, du doigt.
 narrateur|Le bateau glisse entre deux dalles.
-narrateur|L'escargot s'écarte, tout lent.
+narrateur|L'escargot s'écarte, très lent.
 enfant-m|Il laisse passer !
-papa|Oui.
 narrateur|Une feuille collée barre le chemin.
-narrateur|Le bateau s'arrête.
-enfant-m|Il est coincé.
-maman|Tu peux le dégager.
+narrateur|Le bateau s'arrête, loin de l'éclat.
+enfant-m|Il est coincé !
+enfant-m|Il n'arrive pas au bout.
+narrateur|Le sourire d'Aniss disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|L'éclat de dalle tremble, puis tient.
+narrateur|Les épaules d'Aniss tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu vois la feuille ?
+enfant-m|Oui, papa.
 narrateur|Aniss cherche autour de la flaque.
 narrateur|Il regarde Chouchou.
 enfant-m|Tu m'aides ?
-copain|Plus tard.
-enfant-m|D'accord.
-papa|La feuille est juste devant.
-narrateur|Le zinc goutte encore une fois.
-narrateur|Le rond tremble, puis s'arrête.</t>
+narrateur|Chouchou serre le torchon.
+narrateur|Elle reste sur la marche.
+enfant-f|Plus tard.
+narrateur|Aniss ouvre la bouche.
+narrateur|Puis il la referme.
+narrateur|Ça serre, dans son ventre.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>pluie,cour</t>
         </is>
       </c>
     </row>
@@ -1416,12 +1433,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou dit plus tard. Que fait Aniss ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Chouchou dit &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;. Que fait Aniss ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Solal invite Maëlys. Que fait-il si Maëlys dit non ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Chouchou dit &lt;emphasis&gt;plus tard&lt;/emphasis&gt;. Que fait Aniss ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1484,7 +1501,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1495,7 +1512,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1510,34 +1527,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>plus tard</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1552,17 +1573,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=chouchou_dit_plus_tard_aniss_accepte; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1595,17 +1616,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Aniss prend une petite brindille. Elle est lisse, un peu mouillée. Il pousse la feuille, tout doux. Le bateau se dégage. Il repart ! Oui. On peut accepter plusieurs réponses. Chouchou reste sur la marche. Il penche la tête. Le deuxième bateau attend au sec. Je mets une voile ? Si tu veux. Chouchou pose une feuille sèche. C'est une voile, sur le papier. Il ne descend pas dans l'eau. Tu as accepté, Aniss. Les deux bateaux glissent. Ils font deux ronds dans la flaque. Ils se croisent ! Ils arrivent au bout. L'escargot a fini sa fissure. Le torchon sent encore l'eau. Tu as fini de les suivre ? Oui, maman.</t>
+          <t>Aniss veut tirer Chouchou vers l'eau. Viens, maintenant ! Chouchou recule d'un pas, sur la marche. Plus tard. Aniss refuse de foncer. Il referme la main. Il écoute la marche, un instant. D'accord. Papa s'accroupit à la même hauteur. Tu restes près de la flaque ? Oui, papa. Maman se baisse aussi. Merci, Aniss. Maman a entendu toute la phrase. Aniss prend une petite brindille. Elle est lisse, un peu mouillée. Il pousse la feuille, sans se presser. Le bateau se dégage. Il repart ! Il glisse ? Oui, papa. Chouchou reste sur la marche. Elle penche la tête. Le deuxième bateau attend au sec. Je mets une voile ? Si tu veux. Chouchou pose une feuille sèche. C'est une voile, sur le papier. Elle ne descend pas dans l'eau. Tu vois la voile ? Oui, papa. Les deux bateaux glissent. Ils font deux ronds dans la flaque. Ils se croisent ! Ils arrivent au bout ? Presque, papa. L'escargot a fini sa fissure. Le ventre d'Aniss se desserre. Tu as les mains froides ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Aniss prend une petite brindille. Elle est lisse, un peu mouillée. Il pousse la feuille, tout doux. Le bateau se dégage. Il repart ! Oui. On peut accepter plusieurs réponses. Chouchou reste sur la marche. Il penche la tête. Le deuxième bateau attend au sec. Je mets une voile ? Si tu veux. Chouchou pose une feuille sèche. C'est une voile, sur le papier. Il ne descend pas dans l'eau. Tu as accepté, Aniss. Les deux bateaux glissent. Ils font deux ronds dans la flaque. Ils se croisent ! Ils arrivent au bout. L'escargot a fini sa fissure. Le torchon sent encore l'eau. Tu as fini de les suivre ? Oui, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss veut tirer Chouchou vers l'eau. Viens, maintenant ! Chouchou recule d'un pas, sur la marche. Plus tard. Aniss refuse de foncer. Il referme la main. Il écoute la marche, un instant. &lt;emphasis level="moderate"&gt;D'accord&lt;/emphasis&gt;. Papa s'accroupit à la même hauteur. Tu restes près de la flaque ? Oui, papa. Maman se baisse aussi. Merci, Aniss. Maman a entendu toute la phrase. Aniss prend une petite brindille. Elle est lisse, un peu mouillée. Il pousse la feuille, sans se presser. Le bateau se dégage. Il repart ! Il glisse ? Oui, papa. Chouchou reste sur la marche. Elle penche la tête. Le deuxième bateau attend au sec. Je mets une voile ? Si tu veux. Chouchou pose une feuille sèche. C'est une voile, sur le papier. Elle ne descend pas dans l'eau. Tu vois la voile ? Oui, papa. Les deux bateaux glissent. Ils font deux ronds dans la flaque. Ils se croisent ! Ils arrivent au bout ? Presque, papa. L'escargot a fini sa fissure. Le ventre d'Aniss se desserre. Tu as les mains froides ? Un peu, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Solal a su &lt;emphasis&gt;proposer&lt;/emphasis&gt;. Il a su accepter plusieurs réponses. [pause]</t>
+          <t>Aniss veut tirer Chouchou vers l'eau. Viens, maintenant ! Chouchou recule d'un pas, sur la marche. Plus tard. Aniss refuse de foncer. Il referme la main. Il écoute la marche, un instant. &lt;emphasis&gt;D'accord&lt;/emphasis&gt;. Papa s'accroupit à la même hauteur. Tu restes près de la flaque ? Oui, papa. Maman se baisse aussi. Merci, Aniss. Maman a entendu toute la phrase. Aniss prend une petite brindille. Elle est lisse, un peu mouillée. Il pousse la feuille, sans se presser. Le bateau se dégage. Il repart ! Il glisse ? Oui, papa. Chouchou reste sur la marche. Elle penche la tête. Le deuxième bateau attend au sec. Je mets une voile ? Si tu veux. Chouchou pose une feuille sèche. C'est une voile, sur le papier. Elle ne descend pas dans l'eau. Tu vois la voile ? Oui, papa. Les deux bateaux glissent. Ils font deux ronds dans la flaque. Ils se croisent ! Ils arrivent au bout ? Presque, papa. L'escargot a fini sa fissure. Le ventre d'Aniss se desserre. Tu as les mains froides ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1652,7 +1673,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1660,10 +1681,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1686,30 +1707,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>D'accord</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1718,10 +1739,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1734,35 +1755,56 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_tirer_dit_d_accord; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Aniss prend une petite brindille.
+          <t>narrateur|Aniss veut tirer Chouchou vers l'eau.
+enfant-m|Viens, maintenant !
+narrateur|Chouchou recule d'un pas, sur la marche.
+enfant-f|Plus tard.
+narrateur|Aniss refuse de foncer.
+narrateur|Il referme la main.
+narrateur|Il écoute la marche, un instant.
+enfant-m|D'accord.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu restes près de la flaque ?
+enfant-m|Oui, papa.
+narrateur|Maman se baisse aussi.
+maman|Merci, Aniss.
+narrateur|Maman a entendu toute la phrase.
+narrateur|Aniss prend une petite brindille.
 narrateur|Elle est lisse, un peu mouillée.
-narrateur|Il pousse la feuille, tout doux.
+narrateur|Il pousse la feuille, sans se presser.
 narrateur|Le bateau se dégage.
 enfant-m|Il repart !
-maman|Oui.
-maman|On peut accepter plusieurs réponses.
+papa|Il glisse ?
+enfant-m|Oui, papa.
 narrateur|Chouchou reste sur la marche.
-narrateur|Il penche la tête.
+narrateur|Elle penche la tête.
 narrateur|Le deuxième bateau attend au sec.
-copain|Je mets une voile ?
+enfant-f|Je mets une voile ?
 enfant-m|Si tu veux.
 narrateur|Chouchou pose une feuille sèche.
 narrateur|C'est une voile, sur le papier.
-narrateur|Il ne descend pas dans l'eau.
-maman|Tu as accepté, Aniss.
+narrateur|Elle ne descend pas dans l'eau.
+papa|Tu vois la voile ?
+enfant-m|Oui, papa.
 narrateur|Les deux bateaux glissent.
 narrateur|Ils font deux ronds dans la flaque.
 enfant-m|Ils se croisent !
-papa|Ils arrivent au bout.
+papa|Ils arrivent au bout ?
+enfant-m|Presque, papa.
 narrateur|L'escargot a fini sa fissure.
-narrateur|Le torchon sent encore l'eau.
-maman|Tu as fini de les suivre ?
-enfant-m|Oui, maman.</t>
+narrateur|Le ventre d'Aniss se desserre.
+maman|Tu as les mains froides ?
+enfant-m|Un peu, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>flaque,bateaux</t>
         </is>
       </c>
     </row>
@@ -1789,17 +1831,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On pose les bateaux au soleil ? Oui. Aniss pose un bateau sur le rebord. Chouchou pose l'autre. Le papier sèche un peu. Tu as fini de poser les bateaux ? Oui, papa. Les chaussettes de Chouchou sont sèches. Les miennes sont un peu mouillées. On les change après. La cour redevient calme. L'escargot est encore là. Il avance toujours. Tout lent.</t>
+          <t>Aniss veut les deux bateaux, d'un coup. Tous les deux, jusqu'à l'éclat ! Il pousse trop vite. Les bateaux se cognent. L'un tourne, loin de la dalle. Oh. La voile se couche. Il n'arrive pas ! Aniss avance la main. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Aniss observe la flaque. Il écoute le zinc, une goutte. Au bout, un éclat de dalle luit. Là, sur la dalle. Aniss tient la brindille des deux mains. La brindille est froide, un peu lisse. Elle est froide, papa. Tu le guides jusqu'à l'éclat ? Oui, papa. On avance ? Oui, maman. Aniss pousse sans se presser. Le bateau glisse vers la dalle. L'air froid revient sur les joues. Chouchou souffle, depuis la marche. Fffff. La voile se relève un peu. Il arrive. On marche. Le papier touche l'éclat, tout au bout.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On pose les bateaux au soleil ? Oui. Aniss pose un bateau sur le rebord. Chouchou pose l'autre. Le papier sèche un peu. Tu as fini de poser les bateaux ? Oui, papa. Les chaussettes de Chouchou sont sèches. Les miennes sont un peu mouillées. On les change après. La cour redevient calme. L'escargot est encore là. Il avance toujours. Tout lent.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss veut les deux bateaux, d'un coup. Tous les deux, jusqu'à l'éclat ! Il pousse trop vite. Les bateaux se cognent. L'un tourne, loin de la dalle. Oh. La voile se couche. Il n'arrive pas ! Aniss avance la main. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Aniss observe la flaque. Il écoute le zinc, une goutte. Au bout, un &lt;emphasis level="moderate"&gt;éclat de dalle&lt;/emphasis&gt; luit. Là, sur la dalle. Aniss tient la brindille des deux mains. La brindille est froide, un peu lisse. Elle est froide, papa. Tu le guides jusqu'à l'éclat ? Oui, papa. On avance ? Oui, maman. Aniss pousse sans se presser. Le bateau glisse vers la dalle. L'air froid revient sur les joues. Chouchou souffle, depuis la marche. Fffff. La voile se relève un peu. Il arrive. On marche. Le papier touche l'éclat, tout au bout.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman range le seau. Solal donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Aniss veut les deux bateaux, d'un coup. Tous les deux, jusqu'à l'éclat ! Il pousse trop vite. Les bateaux se cognent. L'un tourne, loin de la dalle. Oh. La voile se couche. Il n'arrive pas ! Aniss avance la main. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Aniss observe la flaque. Il écoute le zinc, une goutte. Au bout, un &lt;emphasis&gt;éclat de dalle&lt;/emphasis&gt; luit. Là, sur la dalle. Aniss tient la brindille des deux mains. La brindille est froide, un peu lisse. Elle est froide, papa. Tu le guides jusqu'à l'éclat ? Oui, papa. On avance ? Oui, maman. Aniss pousse sans se presser. Le bateau glisse vers la dalle. L'air froid revient sur les joues. Chouchou souffle, depuis la marche. Fffff. La voile se relève un peu. Il arrive. On marche. Le papier touche l'éclat, tout au bout. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1846,7 +1888,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1854,10 +1896,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1880,30 +1922,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de dalle</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1912,10 +1954,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1926,28 +1968,50 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=deux_bateaux_trop_vite_il_observe_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On pose les bateaux au soleil ?
-enfant-m|Oui.
-narrateur|Aniss pose un bateau sur le rebord.
-narrateur|Chouchou pose l'autre.
-narrateur|Le papier sèche un peu.
-papa|Tu as fini de poser les bateaux ?
+          <t>narrateur|Aniss veut les deux bateaux, d'un coup.
+enfant-m|Tous les deux, jusqu'à l'éclat !
+narrateur|Il pousse trop vite.
+narrateur|Les bateaux se cognent.
+narrateur|L'un tourne, loin de la dalle.
+enfant-m|Oh.
+narrateur|La voile se couche.
+enfant-m|Il n'arrive pas !
+narrateur|Aniss avance la main.
+narrateur|Puis il s'arrête net.
+enfant-m|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Aniss observe la flaque.
+narrateur|Il écoute le zinc, une goutte.
+narrateur|Au bout, un éclat de dalle luit.
+enfant-m|Là, sur la dalle.
+narrateur|Aniss tient la brindille des deux mains.
+narrateur|La brindille est froide, un peu lisse.
+enfant-m|Elle est froide, papa.
+papa|Tu le guides jusqu'à l'éclat ?
 enfant-m|Oui, papa.
-maman|Les chaussettes de Chouchou sont sèches.
-enfant-m|Les miennes sont un peu mouillées.
-maman|On les change après.
-narrateur|La cour redevient calme.
-narrateur|L'escargot est encore là.
-papa|Il avance toujours.
-enfant-m|Tout lent.</t>
+maman|On avance ?
+enfant-m|Oui, maman.
+narrateur|Aniss pousse sans se presser.
+narrateur|Le bateau glisse vers la dalle.
+narrateur|L'air froid revient sur les joues.
+narrateur|Chouchou souffle, depuis la marche.
+enfant-f|Fffff.
+narrateur|La voile se relève un peu.
+enfant-m|Il arrive.
+papa|On marche.
+narrateur|Le papier touche l'éclat, tout au bout.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>flaque,zinc</t>
         </is>
       </c>
     </row>
@@ -1974,17 +2038,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Mes bateaux ont couru. Chouchou a regardé. Bravo, Aniss. Le rebord a deux bateaux. Le zinc ne goutte plus.</t>
+          <t>Mes bateaux ont couru, papa. Tu les vois, sur le rebord ? Oui, comme tout à l'heure. Aniss pose un bateau sur le rebord. Chouchou pose l'autre. Le papier sèche un peu. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur la dalle. On est bien, ici. Mes chaussettes sont sèches. Les miennes sont un peu mouillées. On les change après ? Oui, maman. Une goutte quitte le zinc. Elle fait un rond dans la flaque. On le voit, maman. Tu le vois sur la dalle ? Oui, l'éclat. Le soir reste dans l'air. Au bout de la flaque, l'éclat de dalle tient.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Mes bateaux ont couru. Chouchou a regardé. Bravo, Aniss. Le rebord a deux bateaux. Le zinc ne goutte plus.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mes bateaux ont couru, papa. Tu les vois, sur le rebord ? Oui, comme tout à l'heure. Aniss pose un bateau sur le rebord. Chouchou pose l'autre. Le papier sèche un peu. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur la dalle. On est bien, ici. Mes chaussettes sont sèches. Les miennes sont un peu mouillées. On les change après ? Oui, maman. Une goutte quitte le zinc. Elle fait un rond dans la flaque. On le voit, maman. Tu le vois sur la dalle ? Oui, l'éclat. Le soir reste dans l'air. Au bout de la flaque, l'&lt;emphasis level="moderate"&gt;éclat de dalle&lt;/emphasis&gt; tient.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mes bateaux ont couru, papa. Tu les vois, sur le rebord ? Oui, comme tout à l'heure. Aniss pose un bateau sur le rebord. Chouchou pose l'autre. Le papier sèche un peu. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur la dalle. On est bien, ici. Mes chaussettes sont sèches. Les miennes sont un peu mouillées. On les change après ? Oui, maman. Une goutte quitte le zinc. Elle fait un rond dans la flaque. On le voit, maman. Tu le vois sur la dalle ? Oui, l'éclat. Le soir reste dans l'air. Au bout de la flaque, l'&lt;emphasis&gt;éclat de dalle&lt;/emphasis&gt; tient.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2031,15 +2095,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2051,12 +2115,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2065,17 +2129,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de dalle</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2084,11 +2152,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2097,28 +2165,53 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_au_bout_de_la_flaque; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|Mes bateaux ont couru.
-enfant-m|Chouchou a regardé.
-maman|Bravo, Aniss.
-papa|Le rebord a deux bateaux.
-narrateur|Le zinc ne goutte plus.</t>
+          <t>enfant-m|Mes bateaux ont couru, papa.
+papa|Tu les vois, sur le rebord ?
+enfant-m|Oui, comme tout à l'heure.
+narrateur|Aniss pose un bateau sur le rebord.
+narrateur|Chouchou pose l'autre.
+narrateur|Le papier sèche un peu.
+enfant-m|Comme tout à l'heure, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur la dalle.
+maman|On est bien, ici.
+enfant-f|Mes chaussettes sont sèches.
+enfant-m|Les miennes sont un peu mouillées.
+maman|On les change après ?
+enfant-m|Oui, maman.
+narrateur|Une goutte quitte le zinc.
+narrateur|Elle fait un rond dans la flaque.
+enfant-m|On le voit, maman.
+maman|Tu le vois sur la dalle ?
+enfant-m|Oui, l'éclat.
+narrateur|Le soir reste dans l'air.
+narrateur|Au bout de la flaque, l'éclat de dalle tient.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>zinc,dalles</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2217,6 +2310,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>